<commit_message>
Actualización módulos POS, veterinaria, reportes y plantilla inventario
</commit_message>
<xml_diff>
--- a/plantilla_inventario_POSmaster.xlsx
+++ b/plantilla_inventario_POSmaster.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MIS APP\POSmaster\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C67D9CCA-4AEC-4399-B191-7BE8663E3CFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF26E3F5-E230-4F45-958E-FE9A38314F6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="3180" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Productos" sheetId="1" r:id="rId1"/>
@@ -577,13 +577,13 @@
         <v>30</v>
       </c>
       <c r="G2">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="H2">
-        <v>189000</v>
+        <v>100000</v>
       </c>
       <c r="I2">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="J2">
         <v>1</v>

</xml_diff>